<commit_message>
refactor: renombrar módulos 01-06 → 1-7 y agregar pipeline completo
Reestructuración del pipeline de cobranza JASS:
- Módulos renombrados sin ceros (01_lecturas→1_lecturas, etc.)
- Nuevos módulos: 2_planilla, 5_cobranza, 5b_validacion, 6_corte, 6b_override, 7_cierre
- 3_boletas: enriquecimiento integrado como submódulo
- 4_pagos: efectivo y yape separados con motor_matching completo
- .gitignore actualizado: rutas nuevas, .venv, outputs minúscula
- docs: skill_tracker, metodología v2.9, ADRs, reportes aprendizaje 2026-05 a 06
- shared: planilla y reportes junio 2026

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shared/blancos_acumulados.xlsx
+++ b/shared/blancos_acumulados.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,11 +94,6 @@
       <name val="Courier New"/>
       <color rgb="00A32D2D"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="007D6608"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="12">
@@ -257,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -316,12 +311,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -687,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -708,7 +697,6 @@
     <col width="30" customWidth="1" min="16" max="16"/>
     <col width="1" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -745,14 +733,13 @@
       <c r="O1" s="21" t="n"/>
       <c r="P1" s="20" t="n"/>
       <c r="Q1" s="2" t="inlineStr"/>
-      <c r="R1" s="22" t="inlineStr">
-        <is>
-          <t>¿Ya se aplicó?</t>
-        </is>
-      </c>
-      <c r="S1" s="20" t="n"/>
+      <c r="R1" s="6" t="inlineStr">
+        <is>
+          <t>¿YA SE APLICÓ?</t>
+        </is>
+      </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>MES</t>
@@ -825,11 +812,6 @@
       <c r="R2" s="6" t="inlineStr">
         <is>
           <t>ESTADO</t>
-        </is>
-      </c>
-      <c r="S2" s="23" t="inlineStr">
-        <is>
-          <t>MES_APLICADO</t>
         </is>
       </c>
     </row>
@@ -840,8 +822,8 @@
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="12" t="inlineStr"/>
-      <c r="D3" s="13" t="inlineStr"/>
+      <c r="C3" s="12" t="n"/>
+      <c r="D3" s="13" t="n"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr">
         <is>
@@ -853,21 +835,21 @@
           <t>Juliana Med*</t>
         </is>
       </c>
-      <c r="H3" s="14" t="inlineStr"/>
+      <c r="H3" s="14" t="n"/>
       <c r="I3" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="J3" s="16" t="inlineStr"/>
+      <c r="J3" s="16" t="n"/>
       <c r="K3" s="14" t="inlineStr">
         <is>
           <t>02/05/2026 13:31:48</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="17" t="inlineStr"/>
-      <c r="N3" s="17" t="inlineStr"/>
-      <c r="O3" s="18" t="inlineStr"/>
-      <c r="P3" s="18" t="inlineStr"/>
+      <c r="M3" s="17" t="n"/>
+      <c r="N3" s="17" t="n"/>
+      <c r="O3" s="18" t="n"/>
+      <c r="P3" s="18" t="n"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="19" t="inlineStr">
         <is>
@@ -875,12 +857,95 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>TE PAGÓ</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>PLIN - ANALI QUINECHE</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n"/>
+      <c r="I4" s="15" t="n">
+        <v>103</v>
+      </c>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>05/06/2026 17:34:08</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="17" t="n"/>
+      <c r="N4" s="17" t="n"/>
+      <c r="O4" s="18" t="n"/>
+      <c r="P4" s="18" t="n"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="19" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="12" t="inlineStr"/>
+      <c r="D5" s="13" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>TE PAGÓ</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Sthefany Cre*</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr"/>
+      <c r="I5" s="15" t="n">
+        <v>58</v>
+      </c>
+      <c r="J5" s="16" t="inlineStr"/>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>10/06/2026 12:52:36</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="17" t="inlineStr"/>
+      <c r="N5" s="17" t="inlineStr"/>
+      <c r="O5" s="18" t="inlineStr"/>
+      <c r="P5" s="18" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="19" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="M1:P1"/>
     <mergeCell ref="F1:K1"/>
-    <mergeCell ref="R1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(shared): overlays del ledger + datos del ciclo julio-agosto
Entran a git los overlays que hasta hoy vivian solo en disco: abonos_rezagados,
reasignaciones_aplicacion, devoluciones_aplicadas, exoneraciones_multa,
deuda_correcciones, reidentificacion, blancos_efectivo, aportes_tanque_manuales
y los backups del ledger. Sin ellos el estado del pueblo no es reproducible.

Suma los README de 5_cobranza y 5b_validacion, y el ciclo activo al dia.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shared/blancos_acumulados.xlsx
+++ b/shared/blancos_acumulados.xlsx
@@ -154,7 +154,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -204,11 +204,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -265,6 +309,8 @@
     <xf numFmtId="0" fontId="13" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -665,18 +711,27 @@
           <t>¿QUIÉN ES?</t>
         </is>
       </c>
+      <c r="D1" s="20" t="n"/>
       <c r="E1" s="2" t="inlineStr"/>
       <c r="F1" s="4" t="inlineStr">
         <is>
           <t>¿QUÉ HIZO EL BANCO?</t>
         </is>
       </c>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="21" t="n"/>
+      <c r="I1" s="21" t="n"/>
+      <c r="J1" s="21" t="n"/>
+      <c r="K1" s="20" t="n"/>
       <c r="L1" s="2" t="inlineStr"/>
       <c r="M1" s="5" t="inlineStr">
         <is>
           <t>¿CÓMO SE IDENTIFICÓ?</t>
         </is>
       </c>
+      <c r="N1" s="21" t="n"/>
+      <c r="O1" s="21" t="n"/>
+      <c r="P1" s="20" t="n"/>
       <c r="Q1" s="2" t="inlineStr"/>
       <c r="R1" s="6" t="inlineStr">
         <is>
@@ -875,14 +930,24 @@
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
+      <c r="M5" s="17" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N5" s="17" t="n">
+        <v>8</v>
+      </c>
       <c r="O5" s="18" t="n"/>
-      <c r="P5" s="18" t="n"/>
+      <c r="P5" s="18" t="inlineStr">
+        <is>
+          <t>Identificado a E-8 (Gertrudes Vidal Gonzales) - confirmado por la usuaria. Cubre exacto su deuda de junio (5 consumo + 3 mant + 50 multa = 58, cero pagos registrados ese mes).</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="19" t="inlineStr">
         <is>
-          <t>pendiente</t>
+          <t>aplicado</t>
         </is>
       </c>
     </row>

</xml_diff>